<commit_message>
Align ownership tab to Owner PDG / DNC Developer framework
Replace the lean-team tab with a responsibility-column legend (D-G:
Owner PDG and DNC Developer lead/secondary) plus the 6-person team
mapped as the Owner PDG staffing side.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXuE4neB3C73XNW19v71hM
</commit_message>
<xml_diff>
--- a/docs/Project_Oversight_Matrix.xlsx
+++ b/docs/Project_Oversight_Matrix.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Oversight Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Team Ownership" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Responsibility &amp; Ownership" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Oversight Matrix'!$A$4:$H$90</definedName>
@@ -50,7 +50,7 @@
       <color rgb="001F3864"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5496"/>
       </patternFill>
     </fill>
   </fills>
@@ -127,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +157,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1968,50 +1980,153 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Lean Team — Ownership by Broad Category</t>
+          <t>Responsibility Framework &amp; Ownership Key</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Team Member</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Matrix Responsibility Columns (D–G) — What They Mean</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Matrix Column</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>D — Lead Responsibility – Owner PDG</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Owner PDG</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Owner's project team (PDG) holds primary accountability: drives, decides, and owns the outcome.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>E — Secondary Responsibility – Owner PDG</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Owner PDG</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Owner PDG supporting / backup role: reviews, contributes, or covers when the lead is unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>F — Lead Responsibility – DNC Developer</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>DNC Developer</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>DNC Developer holds primary accountability for executing and delivering the item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>G — Secondary Responsibility – DNC Developer</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>DNC Developer</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>DNC Developer supporting / backup role: assists or steps in behind the developer lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Owner PDG — Lean Team Staffing by Oversight Area</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n"/>
+      <c r="C10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>PDG Team Member</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Primary Domains</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Oversight Areas Owned (from Matrix)</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="11" t="inlineStr">
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Cost, Change Orders, Contracts</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>2. Budget / Cost Control
 4. Change Management
@@ -2019,18 +2134,18 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Person 2</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Schedule, Procurement, Logistics</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>3. Schedule Management
 10. Procurement &amp; Long Lead Items
@@ -2038,18 +2153,18 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Person 3</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Quality, Design, Commissioning</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>5. Scope Control
 6. Design Coordination &amp; Completion
@@ -2059,36 +2174,36 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Person 4</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Site Operations — General Trades</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>8. Safety Performance
 9. Labor &amp; Workforce Management</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Person 5</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Site Operations — MEP, FA, FP, Security</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>12. MEP &amp; Systems Integration
 14. Casino-Specific Systems / Interface
@@ -2096,18 +2211,18 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Person 6</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Risk, Reporting, Governance</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>1. Governance &amp; Decision Framework
 16. Reporting &amp; Transparency
@@ -2116,17 +2231,19 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Note: Categories 8 &amp; 9 (Safety, Labor) sit with Site Ops (P4). MEP/Casino systems &amp; ESG (12, 14, 18) sit with P5. Adjust ownership to match your final org chart.</t>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Notes: (1) The 6-person lean team staffs the Owner PDG side (matrix columns D–E). Populate columns F–G with the DNC Developer counterparts. (2) Safety &amp; Labor (8, 9) sit with Site Ops (P4); MEP/Casino systems &amp; ESG (12, 14, 18) with P5. Adjust to match the final org chart.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A10:C10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Match workbook color scheme to CM Interview deck (navy + gold)
Retheme to the deck palette: deep navy headers (12263A), gold section
bands (C8A04B), grey-blue grid lines, light-grey alt rows, and
Calibri Light titles.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXuE4neB3C73XNW19v71hM
</commit_message>
<xml_diff>
--- a/docs/Project_Oversight_Matrix.xlsx
+++ b/docs/Project_Oversight_Matrix.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,14 +29,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Calibri Light"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="0012263A"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00808080"/>
+      <color rgb="005A6570"/>
       <sz val="10"/>
     </font>
     <font>
@@ -47,7 +47,13 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="0012263A"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="0012263A"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -59,17 +65,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="0012263A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5FB"/>
+        <fgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E5496"/>
+        <fgColor rgb="00C8A04B"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,21 +89,21 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </bottom>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </left>
       <right/>
       <top/>
@@ -106,10 +112,10 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </right>
       <top/>
       <bottom/>
@@ -117,14 +123,14 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00C9D2DE"/>
       </bottom>
       <diagonal/>
     </border>
@@ -159,7 +165,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>

</xml_diff>

<commit_message>
Apply gold category bands to matrix page for scheme parity
Add gold (C8A04B) category bands to the Oversight Matrix page so the
navy + gold scheme appears consistently on both sheets.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXuE4neB3C73XNW19v71hM
</commit_message>
<xml_diff>
--- a/docs/Project_Oversight_Matrix.xlsx
+++ b/docs/Project_Oversight_Matrix.xlsx
@@ -70,12 +70,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4F6F8"/>
+        <fgColor rgb="00C8A04B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8A04B"/>
+        <fgColor rgb="00F4F6F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,27 +145,27 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -620,115 +620,115 @@
           <t>Clear authority matrix (Owner Teams / CM / Designer)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="n"/>
-      <c r="B6" s="7" t="n"/>
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="8" t="n"/>
       <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Escalation paths and approval timelines</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="9" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Executive steering cadence</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Budget / Cost Control</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>GMP vs. Budget forecast</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="11" t="inlineStr"/>
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n"/>
-      <c r="B9" s="7" t="n"/>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Cost-to-complete and contingency drawdown</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="9" t="inlineStr"/>
-      <c r="H9" s="11" t="inlineStr"/>
+      <c r="D9" s="11" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr"/>
+      <c r="G9" s="11" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="n"/>
-      <c r="B10" s="7" t="n"/>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Trend logs and forecast accuracy</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr"/>
-      <c r="E10" s="9" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr"/>
-      <c r="H10" s="11" t="inlineStr"/>
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="n"/>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>Cashflow</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr"/>
-      <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
-      <c r="G11" s="9" t="inlineStr"/>
-      <c r="H11" s="11" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr"/>
+      <c r="H11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="8" t="n"/>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="9" t="n"/>
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>Lender interface</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr"/>
-      <c r="H12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -744,143 +744,143 @@
           <t>Critical path tracking</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
-      <c r="B14" s="7" t="n"/>
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
       <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Milestone adherence</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="n"/>
-      <c r="B15" s="7" t="n"/>
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
       <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Recovery schedule and plans for slippage</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n"/>
-      <c r="B16" s="8" t="n"/>
+      <c r="A16" s="9" t="n"/>
+      <c r="B16" s="9" t="n"/>
       <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Owner scheduling consultant</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n">
+      <c r="A17" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Change Management</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>Change order procedure: determination of need, entitlement, fair and reasonable pricing</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr"/>
-      <c r="F17" s="9" t="inlineStr"/>
-      <c r="G17" s="9" t="inlineStr"/>
-      <c r="H17" s="11" t="inlineStr"/>
+      <c r="D17" s="11" t="inlineStr"/>
+      <c r="E17" s="11" t="inlineStr"/>
+      <c r="F17" s="11" t="inlineStr"/>
+      <c r="G17" s="11" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="n"/>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>CO pipeline (approved vs. pending)</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr"/>
-      <c r="E18" s="9" t="inlineStr"/>
-      <c r="F18" s="9" t="inlineStr"/>
-      <c r="G18" s="9" t="inlineStr"/>
-      <c r="H18" s="11" t="inlineStr"/>
+      <c r="D18" s="11" t="inlineStr"/>
+      <c r="E18" s="11" t="inlineStr"/>
+      <c r="F18" s="11" t="inlineStr"/>
+      <c r="G18" s="11" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="n"/>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>Reason codes / root causes (design gaps, owner changes, unforeseen field conditions)</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr"/>
-      <c r="E19" s="9" t="inlineStr"/>
-      <c r="F19" s="9" t="inlineStr"/>
-      <c r="G19" s="9" t="inlineStr"/>
-      <c r="H19" s="11" t="inlineStr"/>
+      <c r="D19" s="11" t="inlineStr"/>
+      <c r="E19" s="11" t="inlineStr"/>
+      <c r="F19" s="11" t="inlineStr"/>
+      <c r="G19" s="11" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="7" t="n"/>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Cost / schedule impact tracking</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr"/>
-      <c r="E20" s="9" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr"/>
-      <c r="G20" s="9" t="inlineStr"/>
-      <c r="H20" s="11" t="inlineStr"/>
+      <c r="D20" s="11" t="inlineStr"/>
+      <c r="E20" s="11" t="inlineStr"/>
+      <c r="F20" s="11" t="inlineStr"/>
+      <c r="G20" s="11" t="inlineStr"/>
+      <c r="H20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="n"/>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>Requests: RFI, RFP, COR, CCD</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr"/>
-      <c r="E21" s="9" t="inlineStr"/>
-      <c r="F21" s="9" t="inlineStr"/>
-      <c r="G21" s="9" t="inlineStr"/>
-      <c r="H21" s="11" t="inlineStr"/>
+      <c r="D21" s="11" t="inlineStr"/>
+      <c r="E21" s="11" t="inlineStr"/>
+      <c r="F21" s="11" t="inlineStr"/>
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="A22" s="9" t="n"/>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>Claims &amp; disputes</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr"/>
-      <c r="E22" s="9" t="inlineStr"/>
-      <c r="F22" s="9" t="inlineStr"/>
-      <c r="G22" s="9" t="inlineStr"/>
-      <c r="H22" s="11" t="inlineStr"/>
+      <c r="D22" s="11" t="inlineStr"/>
+      <c r="E22" s="11" t="inlineStr"/>
+      <c r="F22" s="11" t="inlineStr"/>
+      <c r="G22" s="11" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -896,129 +896,129 @@
           <t>Alignment between design intent and construction scope</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr"/>
+      <c r="E23" s="7" t="inlineStr"/>
+      <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr"/>
       <c r="H23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n"/>
-      <c r="B24" s="7" t="n"/>
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Prevention of scope creep</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr"/>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
+      <c r="A25" s="9" t="n"/>
+      <c r="B25" s="9" t="n"/>
       <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Trade scope completeness</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr"/>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="7" t="inlineStr"/>
+      <c r="G25" s="7" t="inlineStr"/>
       <c r="H25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n">
+      <c r="A26" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Design Coordination &amp; Completion</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>% design complete (IFC quality)</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr"/>
-      <c r="E26" s="9" t="inlineStr"/>
-      <c r="F26" s="9" t="inlineStr"/>
-      <c r="G26" s="9" t="inlineStr"/>
-      <c r="H26" s="11" t="inlineStr"/>
+      <c r="D26" s="11" t="inlineStr"/>
+      <c r="E26" s="11" t="inlineStr"/>
+      <c r="F26" s="11" t="inlineStr"/>
+      <c r="G26" s="11" t="inlineStr"/>
+      <c r="H26" s="10" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>Coordination issues (MEP clashes, architecture)</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr"/>
-      <c r="E27" s="9" t="inlineStr"/>
-      <c r="F27" s="9" t="inlineStr"/>
-      <c r="G27" s="9" t="inlineStr"/>
-      <c r="H27" s="11" t="inlineStr"/>
+      <c r="D27" s="11" t="inlineStr"/>
+      <c r="E27" s="11" t="inlineStr"/>
+      <c r="F27" s="11" t="inlineStr"/>
+      <c r="G27" s="11" t="inlineStr"/>
+      <c r="H27" s="10" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="n"/>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>Architect / engineer responsiveness</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr"/>
-      <c r="E28" s="9" t="inlineStr"/>
-      <c r="F28" s="9" t="inlineStr"/>
-      <c r="G28" s="9" t="inlineStr"/>
-      <c r="H28" s="11" t="inlineStr"/>
+      <c r="D28" s="11" t="inlineStr"/>
+      <c r="E28" s="11" t="inlineStr"/>
+      <c r="F28" s="11" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr"/>
+      <c r="H28" s="10" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="n"/>
-      <c r="B29" s="7" t="n"/>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Interface and coordination with developer</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr"/>
-      <c r="E29" s="9" t="inlineStr"/>
-      <c r="F29" s="9" t="inlineStr"/>
-      <c r="G29" s="9" t="inlineStr"/>
-      <c r="H29" s="11" t="inlineStr"/>
+      <c r="D29" s="11" t="inlineStr"/>
+      <c r="E29" s="11" t="inlineStr"/>
+      <c r="F29" s="11" t="inlineStr"/>
+      <c r="G29" s="11" t="inlineStr"/>
+      <c r="H29" s="10" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="7" t="n"/>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>Coordination with owner consultants</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr"/>
-      <c r="E30" s="9" t="inlineStr"/>
-      <c r="F30" s="9" t="inlineStr"/>
-      <c r="G30" s="9" t="inlineStr"/>
-      <c r="H30" s="11" t="inlineStr"/>
+      <c r="D30" s="11" t="inlineStr"/>
+      <c r="E30" s="11" t="inlineStr"/>
+      <c r="F30" s="11" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr"/>
+      <c r="H30" s="10" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="n"/>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="A31" s="9" t="n"/>
+      <c r="B31" s="9" t="n"/>
+      <c r="C31" s="10" t="inlineStr">
         <is>
           <t>Pay applications</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr"/>
-      <c r="E31" s="9" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr"/>
-      <c r="G31" s="9" t="inlineStr"/>
-      <c r="H31" s="11" t="inlineStr"/>
+      <c r="D31" s="11" t="inlineStr"/>
+      <c r="E31" s="11" t="inlineStr"/>
+      <c r="F31" s="11" t="inlineStr"/>
+      <c r="G31" s="11" t="inlineStr"/>
+      <c r="H31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -1034,129 +1034,129 @@
           <t>QA/QC program effectiveness</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr"/>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
+      <c r="D32" s="7" t="inlineStr"/>
+      <c r="E32" s="7" t="inlineStr"/>
+      <c r="F32" s="7" t="inlineStr"/>
+      <c r="G32" s="7" t="inlineStr"/>
       <c r="H32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="7" t="n"/>
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
       <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Inspection results</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr"/>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="D33" s="7" t="inlineStr"/>
+      <c r="E33" s="7" t="inlineStr"/>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="7" t="inlineStr"/>
       <c r="H33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="7" t="n"/>
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
       <c r="C34" s="6" t="inlineStr">
         <is>
           <t>NCNs — Non-Conformance Notices</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr"/>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
+      <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="7" t="inlineStr"/>
+      <c r="F34" s="7" t="inlineStr"/>
+      <c r="G34" s="7" t="inlineStr"/>
       <c r="H34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="n"/>
-      <c r="B35" s="8" t="n"/>
+      <c r="A35" s="9" t="n"/>
+      <c r="B35" s="9" t="n"/>
       <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Mockups and finishes (critical for a casino)</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr"/>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
+      <c r="D35" s="7" t="inlineStr"/>
+      <c r="E35" s="7" t="inlineStr"/>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="7" t="inlineStr"/>
       <c r="H35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n">
+      <c r="A36" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Safety Performance</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>OSHA partnering</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr"/>
-      <c r="E36" s="9" t="inlineStr"/>
-      <c r="F36" s="9" t="inlineStr"/>
-      <c r="G36" s="9" t="inlineStr"/>
-      <c r="H36" s="11" t="inlineStr"/>
+      <c r="D36" s="11" t="inlineStr"/>
+      <c r="E36" s="11" t="inlineStr"/>
+      <c r="F36" s="11" t="inlineStr"/>
+      <c r="G36" s="11" t="inlineStr"/>
+      <c r="H36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
-      <c r="B37" s="7" t="n"/>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="10" t="inlineStr">
         <is>
           <t>Safety culture</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr"/>
-      <c r="E37" s="9" t="inlineStr"/>
-      <c r="F37" s="9" t="inlineStr"/>
-      <c r="G37" s="9" t="inlineStr"/>
-      <c r="H37" s="11" t="inlineStr"/>
+      <c r="D37" s="11" t="inlineStr"/>
+      <c r="E37" s="11" t="inlineStr"/>
+      <c r="F37" s="11" t="inlineStr"/>
+      <c r="G37" s="11" t="inlineStr"/>
+      <c r="H37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
-      <c r="B38" s="7" t="n"/>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>Contractors' safety programs</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr"/>
-      <c r="E38" s="9" t="inlineStr"/>
-      <c r="F38" s="9" t="inlineStr"/>
-      <c r="G38" s="9" t="inlineStr"/>
-      <c r="H38" s="11" t="inlineStr"/>
+      <c r="D38" s="11" t="inlineStr"/>
+      <c r="E38" s="11" t="inlineStr"/>
+      <c r="F38" s="11" t="inlineStr"/>
+      <c r="G38" s="11" t="inlineStr"/>
+      <c r="H38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n"/>
-      <c r="B39" s="7" t="n"/>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>Safety compliance</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr"/>
-      <c r="E39" s="9" t="inlineStr"/>
-      <c r="F39" s="9" t="inlineStr"/>
-      <c r="G39" s="9" t="inlineStr"/>
-      <c r="H39" s="11" t="inlineStr"/>
+      <c r="D39" s="11" t="inlineStr"/>
+      <c r="E39" s="11" t="inlineStr"/>
+      <c r="F39" s="11" t="inlineStr"/>
+      <c r="G39" s="11" t="inlineStr"/>
+      <c r="H39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="n"/>
-      <c r="B40" s="8" t="n"/>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="A40" s="9" t="n"/>
+      <c r="B40" s="9" t="n"/>
+      <c r="C40" s="10" t="inlineStr">
         <is>
           <t>Safety officer</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr"/>
-      <c r="E40" s="9" t="inlineStr"/>
-      <c r="F40" s="9" t="inlineStr"/>
-      <c r="G40" s="9" t="inlineStr"/>
-      <c r="H40" s="11" t="inlineStr"/>
+      <c r="D40" s="11" t="inlineStr"/>
+      <c r="E40" s="11" t="inlineStr"/>
+      <c r="F40" s="11" t="inlineStr"/>
+      <c r="G40" s="11" t="inlineStr"/>
+      <c r="H40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -1172,87 +1172,87 @@
           <t>Labor availability (especially skilled trades)</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
-      <c r="G41" s="4" t="inlineStr"/>
+      <c r="D41" s="7" t="inlineStr"/>
+      <c r="E41" s="7" t="inlineStr"/>
+      <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr"/>
       <c r="H41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="n"/>
-      <c r="B42" s="7" t="n"/>
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
       <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Reporting: monthly manpower reports</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="4" t="inlineStr"/>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="4" t="inlineStr"/>
+      <c r="D42" s="7" t="inlineStr"/>
+      <c r="E42" s="7" t="inlineStr"/>
+      <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
       <c r="H42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="n"/>
+      <c r="A43" s="9" t="n"/>
+      <c r="B43" s="9" t="n"/>
       <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Union dynamics (if applicable in Colorado markets)</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr"/>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="D43" s="7" t="inlineStr"/>
+      <c r="E43" s="7" t="inlineStr"/>
+      <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr"/>
       <c r="H43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="n">
+      <c r="A44" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>Procurement &amp; Long Lead Items</t>
         </is>
       </c>
-      <c r="C44" s="11" t="inlineStr">
+      <c r="C44" s="10" t="inlineStr">
         <is>
           <t>Key materials (steel, curtain wall, gaming systems, elevators)</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr"/>
-      <c r="E44" s="9" t="inlineStr"/>
-      <c r="F44" s="9" t="inlineStr"/>
-      <c r="G44" s="9" t="inlineStr"/>
-      <c r="H44" s="11" t="inlineStr"/>
+      <c r="D44" s="11" t="inlineStr"/>
+      <c r="E44" s="11" t="inlineStr"/>
+      <c r="F44" s="11" t="inlineStr"/>
+      <c r="G44" s="11" t="inlineStr"/>
+      <c r="H44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="n"/>
-      <c r="B45" s="7" t="n"/>
-      <c r="C45" s="11" t="inlineStr">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>Supply chain risk and delays</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr"/>
-      <c r="E45" s="9" t="inlineStr"/>
-      <c r="F45" s="9" t="inlineStr"/>
-      <c r="G45" s="9" t="inlineStr"/>
-      <c r="H45" s="11" t="inlineStr"/>
+      <c r="D45" s="11" t="inlineStr"/>
+      <c r="E45" s="11" t="inlineStr"/>
+      <c r="F45" s="11" t="inlineStr"/>
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="10" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="n"/>
-      <c r="B46" s="8" t="n"/>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="A46" s="9" t="n"/>
+      <c r="B46" s="9" t="n"/>
+      <c r="C46" s="10" t="inlineStr">
         <is>
           <t>Buyout status and savings approach and tracking</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr"/>
-      <c r="E46" s="9" t="inlineStr"/>
-      <c r="F46" s="9" t="inlineStr"/>
-      <c r="G46" s="9" t="inlineStr"/>
-      <c r="H46" s="11" t="inlineStr"/>
+      <c r="D46" s="11" t="inlineStr"/>
+      <c r="E46" s="11" t="inlineStr"/>
+      <c r="F46" s="11" t="inlineStr"/>
+      <c r="G46" s="11" t="inlineStr"/>
+      <c r="H46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -1268,143 +1268,143 @@
           <t>Developer</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="D47" s="7" t="inlineStr"/>
+      <c r="E47" s="7" t="inlineStr"/>
+      <c r="F47" s="7" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr"/>
       <c r="H47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="n"/>
       <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Construction Manager</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="D48" s="7" t="inlineStr"/>
+      <c r="E48" s="7" t="inlineStr"/>
+      <c r="F48" s="7" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
       <c r="H48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
       <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Operator</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr"/>
+      <c r="D49" s="7" t="inlineStr"/>
+      <c r="E49" s="7" t="inlineStr"/>
+      <c r="F49" s="7" t="inlineStr"/>
+      <c r="G49" s="7" t="inlineStr"/>
       <c r="H49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="7" t="n"/>
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="8" t="n"/>
       <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Specialty vendors / consultants</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4" t="inlineStr"/>
-      <c r="G50" s="4" t="inlineStr"/>
+      <c r="D50" s="7" t="inlineStr"/>
+      <c r="E50" s="7" t="inlineStr"/>
+      <c r="F50" s="7" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
       <c r="H50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="n"/>
-      <c r="B51" s="7" t="n"/>
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
       <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Legal interface</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr"/>
+      <c r="D51" s="7" t="inlineStr"/>
+      <c r="E51" s="7" t="inlineStr"/>
+      <c r="F51" s="7" t="inlineStr"/>
+      <c r="G51" s="7" t="inlineStr"/>
       <c r="H51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="8" t="n"/>
-      <c r="B52" s="8" t="n"/>
+      <c r="A52" s="9" t="n"/>
+      <c r="B52" s="9" t="n"/>
       <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Negotiations</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr"/>
-      <c r="E52" s="4" t="inlineStr"/>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr"/>
+      <c r="D52" s="7" t="inlineStr"/>
+      <c r="E52" s="7" t="inlineStr"/>
+      <c r="F52" s="7" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
       <c r="H52" s="6" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="n">
+      <c r="A53" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>MEP &amp; Systems Integration</t>
         </is>
       </c>
-      <c r="C53" s="11" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>Coordination of mechanical, electrical, plumbing</t>
         </is>
       </c>
-      <c r="D53" s="9" t="inlineStr"/>
-      <c r="E53" s="9" t="inlineStr"/>
-      <c r="F53" s="9" t="inlineStr"/>
-      <c r="G53" s="9" t="inlineStr"/>
-      <c r="H53" s="11" t="inlineStr"/>
+      <c r="D53" s="11" t="inlineStr"/>
+      <c r="E53" s="11" t="inlineStr"/>
+      <c r="F53" s="11" t="inlineStr"/>
+      <c r="G53" s="11" t="inlineStr"/>
+      <c r="H53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="n"/>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="11" t="inlineStr">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="10" t="inlineStr">
         <is>
           <t>Co-Gen plant</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr"/>
-      <c r="E54" s="9" t="inlineStr"/>
-      <c r="F54" s="9" t="inlineStr"/>
-      <c r="G54" s="9" t="inlineStr"/>
-      <c r="H54" s="11" t="inlineStr"/>
+      <c r="D54" s="11" t="inlineStr"/>
+      <c r="E54" s="11" t="inlineStr"/>
+      <c r="F54" s="11" t="inlineStr"/>
+      <c r="G54" s="11" t="inlineStr"/>
+      <c r="H54" s="10" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="n"/>
-      <c r="B55" s="7" t="n"/>
-      <c r="C55" s="11" t="inlineStr">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>Specialty systems: gaming, surveillance, IT backbone</t>
         </is>
       </c>
-      <c r="D55" s="9" t="inlineStr"/>
-      <c r="E55" s="9" t="inlineStr"/>
-      <c r="F55" s="9" t="inlineStr"/>
-      <c r="G55" s="9" t="inlineStr"/>
-      <c r="H55" s="11" t="inlineStr"/>
+      <c r="D55" s="11" t="inlineStr"/>
+      <c r="E55" s="11" t="inlineStr"/>
+      <c r="F55" s="11" t="inlineStr"/>
+      <c r="G55" s="11" t="inlineStr"/>
+      <c r="H55" s="10" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="8" t="n"/>
-      <c r="B56" s="8" t="n"/>
-      <c r="C56" s="11" t="inlineStr">
+      <c r="A56" s="9" t="n"/>
+      <c r="B56" s="9" t="n"/>
+      <c r="C56" s="10" t="inlineStr">
         <is>
           <t>Commissioning readiness</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr"/>
-      <c r="E56" s="9" t="inlineStr"/>
-      <c r="F56" s="9" t="inlineStr"/>
-      <c r="G56" s="9" t="inlineStr"/>
-      <c r="H56" s="11" t="inlineStr"/>
+      <c r="D56" s="11" t="inlineStr"/>
+      <c r="E56" s="11" t="inlineStr"/>
+      <c r="F56" s="11" t="inlineStr"/>
+      <c r="G56" s="11" t="inlineStr"/>
+      <c r="H56" s="10" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n">
@@ -1420,115 +1420,115 @@
           <t>Systems testing plans</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
+      <c r="D57" s="7" t="inlineStr"/>
+      <c r="E57" s="7" t="inlineStr"/>
+      <c r="F57" s="7" t="inlineStr"/>
+      <c r="G57" s="7" t="inlineStr"/>
       <c r="H57" s="6" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="7" t="n"/>
-      <c r="B58" s="7" t="n"/>
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
       <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Phased turnover strategy</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="4" t="inlineStr"/>
-      <c r="F58" s="4" t="inlineStr"/>
-      <c r="G58" s="4" t="inlineStr"/>
+      <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="7" t="inlineStr"/>
+      <c r="F58" s="7" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
       <c r="H58" s="6" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="7" t="n"/>
-      <c r="B59" s="7" t="n"/>
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="8" t="n"/>
       <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Owner training and documentation</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr"/>
-      <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="4" t="inlineStr"/>
+      <c r="D59" s="7" t="inlineStr"/>
+      <c r="E59" s="7" t="inlineStr"/>
+      <c r="F59" s="7" t="inlineStr"/>
+      <c r="G59" s="7" t="inlineStr"/>
       <c r="H59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="n"/>
-      <c r="B60" s="8" t="n"/>
+      <c r="A60" s="9" t="n"/>
+      <c r="B60" s="9" t="n"/>
       <c r="C60" s="6" t="inlineStr">
         <is>
           <t>O&amp;M manuals, warranties</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr"/>
-      <c r="F60" s="4" t="inlineStr"/>
-      <c r="G60" s="4" t="inlineStr"/>
+      <c r="D60" s="7" t="inlineStr"/>
+      <c r="E60" s="7" t="inlineStr"/>
+      <c r="F60" s="7" t="inlineStr"/>
+      <c r="G60" s="7" t="inlineStr"/>
       <c r="H60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="9" t="n">
+      <c r="A61" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>Casino-Specific Systems / Interface</t>
         </is>
       </c>
-      <c r="C61" s="11" t="inlineStr">
+      <c r="C61" s="10" t="inlineStr">
         <is>
           <t>Gaming floor integration</t>
         </is>
       </c>
-      <c r="D61" s="9" t="inlineStr"/>
-      <c r="E61" s="9" t="inlineStr"/>
-      <c r="F61" s="9" t="inlineStr"/>
-      <c r="G61" s="9" t="inlineStr"/>
-      <c r="H61" s="11" t="inlineStr"/>
+      <c r="D61" s="11" t="inlineStr"/>
+      <c r="E61" s="11" t="inlineStr"/>
+      <c r="F61" s="11" t="inlineStr"/>
+      <c r="G61" s="11" t="inlineStr"/>
+      <c r="H61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="n"/>
-      <c r="B62" s="7" t="n"/>
-      <c r="C62" s="11" t="inlineStr">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="8" t="n"/>
+      <c r="C62" s="10" t="inlineStr">
         <is>
           <t>Surveillance &amp; security systems (highly regulated)</t>
         </is>
       </c>
-      <c r="D62" s="9" t="inlineStr"/>
-      <c r="E62" s="9" t="inlineStr"/>
-      <c r="F62" s="9" t="inlineStr"/>
-      <c r="G62" s="9" t="inlineStr"/>
-      <c r="H62" s="11" t="inlineStr"/>
+      <c r="D62" s="11" t="inlineStr"/>
+      <c r="E62" s="11" t="inlineStr"/>
+      <c r="F62" s="11" t="inlineStr"/>
+      <c r="G62" s="11" t="inlineStr"/>
+      <c r="H62" s="10" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="7" t="n"/>
-      <c r="B63" s="7" t="n"/>
-      <c r="C63" s="11" t="inlineStr">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="8" t="n"/>
+      <c r="C63" s="10" t="inlineStr">
         <is>
           <t>Food and beverage; retail</t>
         </is>
       </c>
-      <c r="D63" s="9" t="inlineStr"/>
-      <c r="E63" s="9" t="inlineStr"/>
-      <c r="F63" s="9" t="inlineStr"/>
-      <c r="G63" s="9" t="inlineStr"/>
-      <c r="H63" s="11" t="inlineStr"/>
+      <c r="D63" s="11" t="inlineStr"/>
+      <c r="E63" s="11" t="inlineStr"/>
+      <c r="F63" s="11" t="inlineStr"/>
+      <c r="G63" s="11" t="inlineStr"/>
+      <c r="H63" s="10" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="n"/>
-      <c r="B64" s="8" t="n"/>
-      <c r="C64" s="11" t="inlineStr">
+      <c r="A64" s="9" t="n"/>
+      <c r="B64" s="9" t="n"/>
+      <c r="C64" s="10" t="inlineStr">
         <is>
           <t>Hotel</t>
         </is>
       </c>
-      <c r="D64" s="9" t="inlineStr"/>
-      <c r="E64" s="9" t="inlineStr"/>
-      <c r="F64" s="9" t="inlineStr"/>
-      <c r="G64" s="9" t="inlineStr"/>
-      <c r="H64" s="11" t="inlineStr"/>
+      <c r="D64" s="11" t="inlineStr"/>
+      <c r="E64" s="11" t="inlineStr"/>
+      <c r="F64" s="11" t="inlineStr"/>
+      <c r="G64" s="11" t="inlineStr"/>
+      <c r="H64" s="10" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
@@ -1544,157 +1544,157 @@
           <t>Laydown areas and material flow</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr"/>
-      <c r="E65" s="4" t="inlineStr"/>
-      <c r="F65" s="4" t="inlineStr"/>
-      <c r="G65" s="4" t="inlineStr"/>
+      <c r="D65" s="7" t="inlineStr"/>
+      <c r="E65" s="7" t="inlineStr"/>
+      <c r="F65" s="7" t="inlineStr"/>
+      <c r="G65" s="7" t="inlineStr"/>
       <c r="H65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="7" t="n"/>
-      <c r="B66" s="7" t="n"/>
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="8" t="n"/>
       <c r="C66" s="6" t="inlineStr">
         <is>
           <t>Urban / site constraints</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr"/>
-      <c r="E66" s="4" t="inlineStr"/>
-      <c r="F66" s="4" t="inlineStr"/>
-      <c r="G66" s="4" t="inlineStr"/>
+      <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="7" t="inlineStr"/>
+      <c r="F66" s="7" t="inlineStr"/>
+      <c r="G66" s="7" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="8" t="n"/>
-      <c r="B67" s="8" t="n"/>
+      <c r="A67" s="9" t="n"/>
+      <c r="B67" s="9" t="n"/>
       <c r="C67" s="6" t="inlineStr">
         <is>
           <t>Sequencing of major trades</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr"/>
-      <c r="E67" s="4" t="inlineStr"/>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="4" t="inlineStr"/>
+      <c r="D67" s="7" t="inlineStr"/>
+      <c r="E67" s="7" t="inlineStr"/>
+      <c r="F67" s="7" t="inlineStr"/>
+      <c r="G67" s="7" t="inlineStr"/>
       <c r="H67" s="6" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="n">
+      <c r="A68" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B68" s="10" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Reporting &amp; Transparency</t>
         </is>
       </c>
-      <c r="C68" s="11" t="inlineStr">
+      <c r="C68" s="10" t="inlineStr">
         <is>
           <t>Cost + fee tracking</t>
         </is>
       </c>
-      <c r="D68" s="9" t="inlineStr"/>
-      <c r="E68" s="9" t="inlineStr"/>
-      <c r="F68" s="9" t="inlineStr"/>
-      <c r="G68" s="9" t="inlineStr"/>
-      <c r="H68" s="11" t="inlineStr"/>
+      <c r="D68" s="11" t="inlineStr"/>
+      <c r="E68" s="11" t="inlineStr"/>
+      <c r="F68" s="11" t="inlineStr"/>
+      <c r="G68" s="11" t="inlineStr"/>
+      <c r="H68" s="10" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="n"/>
-      <c r="B69" s="7" t="n"/>
-      <c r="C69" s="11" t="inlineStr">
+      <c r="A69" s="8" t="n"/>
+      <c r="B69" s="8" t="n"/>
+      <c r="C69" s="10" t="inlineStr">
         <is>
           <t>Accuracy of monthly reports</t>
         </is>
       </c>
-      <c r="D69" s="9" t="inlineStr"/>
-      <c r="E69" s="9" t="inlineStr"/>
-      <c r="F69" s="9" t="inlineStr"/>
-      <c r="G69" s="9" t="inlineStr"/>
-      <c r="H69" s="11" t="inlineStr"/>
+      <c r="D69" s="11" t="inlineStr"/>
+      <c r="E69" s="11" t="inlineStr"/>
+      <c r="F69" s="11" t="inlineStr"/>
+      <c r="G69" s="11" t="inlineStr"/>
+      <c r="H69" s="10" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="7" t="n"/>
-      <c r="B70" s="7" t="n"/>
-      <c r="C70" s="11" t="inlineStr">
+      <c r="A70" s="8" t="n"/>
+      <c r="B70" s="8" t="n"/>
+      <c r="C70" s="10" t="inlineStr">
         <is>
           <t>Schedule, change order / RFI logs</t>
         </is>
       </c>
-      <c r="D70" s="9" t="inlineStr"/>
-      <c r="E70" s="9" t="inlineStr"/>
-      <c r="F70" s="9" t="inlineStr"/>
-      <c r="G70" s="9" t="inlineStr"/>
-      <c r="H70" s="11" t="inlineStr"/>
+      <c r="D70" s="11" t="inlineStr"/>
+      <c r="E70" s="11" t="inlineStr"/>
+      <c r="F70" s="11" t="inlineStr"/>
+      <c r="G70" s="11" t="inlineStr"/>
+      <c r="H70" s="10" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="7" t="n"/>
-      <c r="B71" s="7" t="n"/>
-      <c r="C71" s="11" t="inlineStr">
+      <c r="A71" s="8" t="n"/>
+      <c r="B71" s="8" t="n"/>
+      <c r="C71" s="10" t="inlineStr">
         <is>
           <t>Critical issues</t>
         </is>
       </c>
-      <c r="D71" s="9" t="inlineStr"/>
-      <c r="E71" s="9" t="inlineStr"/>
-      <c r="F71" s="9" t="inlineStr"/>
-      <c r="G71" s="9" t="inlineStr"/>
-      <c r="H71" s="11" t="inlineStr"/>
+      <c r="D71" s="11" t="inlineStr"/>
+      <c r="E71" s="11" t="inlineStr"/>
+      <c r="F71" s="11" t="inlineStr"/>
+      <c r="G71" s="11" t="inlineStr"/>
+      <c r="H71" s="10" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="n"/>
-      <c r="B72" s="7" t="n"/>
-      <c r="C72" s="11" t="inlineStr">
+      <c r="A72" s="8" t="n"/>
+      <c r="B72" s="8" t="n"/>
+      <c r="C72" s="10" t="inlineStr">
         <is>
           <t>Progress photos</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr"/>
-      <c r="E72" s="9" t="inlineStr"/>
-      <c r="F72" s="9" t="inlineStr"/>
-      <c r="G72" s="9" t="inlineStr"/>
-      <c r="H72" s="11" t="inlineStr"/>
+      <c r="D72" s="11" t="inlineStr"/>
+      <c r="E72" s="11" t="inlineStr"/>
+      <c r="F72" s="11" t="inlineStr"/>
+      <c r="G72" s="11" t="inlineStr"/>
+      <c r="H72" s="10" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="n"/>
-      <c r="B73" s="7" t="n"/>
-      <c r="C73" s="11" t="inlineStr">
+      <c r="A73" s="8" t="n"/>
+      <c r="B73" s="8" t="n"/>
+      <c r="C73" s="10" t="inlineStr">
         <is>
           <t>QA/QC</t>
         </is>
       </c>
-      <c r="D73" s="9" t="inlineStr"/>
-      <c r="E73" s="9" t="inlineStr"/>
-      <c r="F73" s="9" t="inlineStr"/>
-      <c r="G73" s="9" t="inlineStr"/>
-      <c r="H73" s="11" t="inlineStr"/>
+      <c r="D73" s="11" t="inlineStr"/>
+      <c r="E73" s="11" t="inlineStr"/>
+      <c r="F73" s="11" t="inlineStr"/>
+      <c r="G73" s="11" t="inlineStr"/>
+      <c r="H73" s="10" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="n"/>
-      <c r="B74" s="7" t="n"/>
-      <c r="C74" s="11" t="inlineStr">
+      <c r="A74" s="8" t="n"/>
+      <c r="B74" s="8" t="n"/>
+      <c r="C74" s="10" t="inlineStr">
         <is>
           <t>Dashboards (KPIs across cost, schedule, safety)</t>
         </is>
       </c>
-      <c r="D74" s="9" t="inlineStr"/>
-      <c r="E74" s="9" t="inlineStr"/>
-      <c r="F74" s="9" t="inlineStr"/>
-      <c r="G74" s="9" t="inlineStr"/>
-      <c r="H74" s="11" t="inlineStr"/>
+      <c r="D74" s="11" t="inlineStr"/>
+      <c r="E74" s="11" t="inlineStr"/>
+      <c r="F74" s="11" t="inlineStr"/>
+      <c r="G74" s="11" t="inlineStr"/>
+      <c r="H74" s="10" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="8" t="n"/>
-      <c r="B75" s="8" t="n"/>
-      <c r="C75" s="11" t="inlineStr">
+      <c r="A75" s="9" t="n"/>
+      <c r="B75" s="9" t="n"/>
+      <c r="C75" s="10" t="inlineStr">
         <is>
           <t>Independent validation (don't rely solely on CM)</t>
         </is>
       </c>
-      <c r="D75" s="9" t="inlineStr"/>
-      <c r="E75" s="9" t="inlineStr"/>
-      <c r="F75" s="9" t="inlineStr"/>
-      <c r="G75" s="9" t="inlineStr"/>
-      <c r="H75" s="11" t="inlineStr"/>
+      <c r="D75" s="11" t="inlineStr"/>
+      <c r="E75" s="11" t="inlineStr"/>
+      <c r="F75" s="11" t="inlineStr"/>
+      <c r="G75" s="11" t="inlineStr"/>
+      <c r="H75" s="10" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
@@ -1710,129 +1710,129 @@
           <t>Local / state approvals</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr"/>
-      <c r="E76" s="4" t="inlineStr"/>
-      <c r="F76" s="4" t="inlineStr"/>
-      <c r="G76" s="4" t="inlineStr"/>
+      <c r="D76" s="7" t="inlineStr"/>
+      <c r="E76" s="7" t="inlineStr"/>
+      <c r="F76" s="7" t="inlineStr"/>
+      <c r="G76" s="7" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="7" t="n"/>
-      <c r="B77" s="7" t="n"/>
+      <c r="A77" s="8" t="n"/>
+      <c r="B77" s="8" t="n"/>
       <c r="C77" s="6" t="inlineStr">
         <is>
           <t>Colorado gaming regs</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr"/>
-      <c r="E77" s="4" t="inlineStr"/>
-      <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="4" t="inlineStr"/>
+      <c r="D77" s="7" t="inlineStr"/>
+      <c r="E77" s="7" t="inlineStr"/>
+      <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="7" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="7" t="n"/>
-      <c r="B78" s="7" t="n"/>
+      <c r="A78" s="8" t="n"/>
+      <c r="B78" s="8" t="n"/>
       <c r="C78" s="6" t="inlineStr">
         <is>
           <t>Building permits</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr"/>
-      <c r="E78" s="4" t="inlineStr"/>
-      <c r="F78" s="4" t="inlineStr"/>
-      <c r="G78" s="4" t="inlineStr"/>
+      <c r="D78" s="7" t="inlineStr"/>
+      <c r="E78" s="7" t="inlineStr"/>
+      <c r="F78" s="7" t="inlineStr"/>
+      <c r="G78" s="7" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="7" t="n"/>
-      <c r="B79" s="7" t="n"/>
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="8" t="n"/>
       <c r="C79" s="6" t="inlineStr">
         <is>
           <t>Inspections and signoffs</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr"/>
-      <c r="E79" s="4" t="inlineStr"/>
-      <c r="F79" s="4" t="inlineStr"/>
-      <c r="G79" s="4" t="inlineStr"/>
+      <c r="D79" s="7" t="inlineStr"/>
+      <c r="E79" s="7" t="inlineStr"/>
+      <c r="F79" s="7" t="inlineStr"/>
+      <c r="G79" s="7" t="inlineStr"/>
       <c r="H79" s="6" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="n"/>
-      <c r="B80" s="8" t="n"/>
+      <c r="A80" s="9" t="n"/>
+      <c r="B80" s="9" t="n"/>
       <c r="C80" s="6" t="inlineStr">
         <is>
           <t>Environmental compliance</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr"/>
-      <c r="E80" s="4" t="inlineStr"/>
-      <c r="F80" s="4" t="inlineStr"/>
-      <c r="G80" s="4" t="inlineStr"/>
+      <c r="D80" s="7" t="inlineStr"/>
+      <c r="E80" s="7" t="inlineStr"/>
+      <c r="F80" s="7" t="inlineStr"/>
+      <c r="G80" s="7" t="inlineStr"/>
       <c r="H80" s="6" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="9" t="n">
+      <c r="A81" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B81" s="10" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr">
         <is>
           <t>Sustainability / ESG (if applicable)</t>
         </is>
       </c>
-      <c r="C81" s="11" t="inlineStr">
+      <c r="C81" s="10" t="inlineStr">
         <is>
           <t>Waste and water management</t>
         </is>
       </c>
-      <c r="D81" s="9" t="inlineStr"/>
-      <c r="E81" s="9" t="inlineStr"/>
-      <c r="F81" s="9" t="inlineStr"/>
-      <c r="G81" s="9" t="inlineStr"/>
-      <c r="H81" s="11" t="inlineStr"/>
+      <c r="D81" s="11" t="inlineStr"/>
+      <c r="E81" s="11" t="inlineStr"/>
+      <c r="F81" s="11" t="inlineStr"/>
+      <c r="G81" s="11" t="inlineStr"/>
+      <c r="H81" s="10" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="7" t="n"/>
-      <c r="B82" s="7" t="n"/>
-      <c r="C82" s="11" t="inlineStr">
+      <c r="A82" s="8" t="n"/>
+      <c r="B82" s="8" t="n"/>
+      <c r="C82" s="10" t="inlineStr">
         <is>
           <t>Mechanical systems</t>
         </is>
       </c>
-      <c r="D82" s="9" t="inlineStr"/>
-      <c r="E82" s="9" t="inlineStr"/>
-      <c r="F82" s="9" t="inlineStr"/>
-      <c r="G82" s="9" t="inlineStr"/>
-      <c r="H82" s="11" t="inlineStr"/>
+      <c r="D82" s="11" t="inlineStr"/>
+      <c r="E82" s="11" t="inlineStr"/>
+      <c r="F82" s="11" t="inlineStr"/>
+      <c r="G82" s="11" t="inlineStr"/>
+      <c r="H82" s="10" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="n"/>
-      <c r="B83" s="7" t="n"/>
-      <c r="C83" s="11" t="inlineStr">
+      <c r="A83" s="8" t="n"/>
+      <c r="B83" s="8" t="n"/>
+      <c r="C83" s="10" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D83" s="9" t="inlineStr"/>
-      <c r="E83" s="9" t="inlineStr"/>
-      <c r="F83" s="9" t="inlineStr"/>
-      <c r="G83" s="9" t="inlineStr"/>
-      <c r="H83" s="11" t="inlineStr"/>
+      <c r="D83" s="11" t="inlineStr"/>
+      <c r="E83" s="11" t="inlineStr"/>
+      <c r="F83" s="11" t="inlineStr"/>
+      <c r="G83" s="11" t="inlineStr"/>
+      <c r="H83" s="10" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="8" t="n"/>
-      <c r="B84" s="8" t="n"/>
-      <c r="C84" s="11" t="inlineStr">
+      <c r="A84" s="9" t="n"/>
+      <c r="B84" s="9" t="n"/>
+      <c r="C84" s="10" t="inlineStr">
         <is>
           <t>Envelope building material selection</t>
         </is>
       </c>
-      <c r="D84" s="9" t="inlineStr"/>
-      <c r="E84" s="9" t="inlineStr"/>
-      <c r="F84" s="9" t="inlineStr"/>
-      <c r="G84" s="9" t="inlineStr"/>
-      <c r="H84" s="11" t="inlineStr"/>
+      <c r="D84" s="11" t="inlineStr"/>
+      <c r="E84" s="11" t="inlineStr"/>
+      <c r="F84" s="11" t="inlineStr"/>
+      <c r="G84" s="11" t="inlineStr"/>
+      <c r="H84" s="10" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -1848,87 +1848,87 @@
           <t>Bonding</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr"/>
-      <c r="E85" s="4" t="inlineStr"/>
-      <c r="F85" s="4" t="inlineStr"/>
-      <c r="G85" s="4" t="inlineStr"/>
+      <c r="D85" s="7" t="inlineStr"/>
+      <c r="E85" s="7" t="inlineStr"/>
+      <c r="F85" s="7" t="inlineStr"/>
+      <c r="G85" s="7" t="inlineStr"/>
       <c r="H85" s="6" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="n"/>
-      <c r="B86" s="7" t="n"/>
+      <c r="A86" s="8" t="n"/>
+      <c r="B86" s="8" t="n"/>
       <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="D86" s="4" t="inlineStr"/>
-      <c r="E86" s="4" t="inlineStr"/>
-      <c r="F86" s="4" t="inlineStr"/>
-      <c r="G86" s="4" t="inlineStr"/>
+      <c r="D86" s="7" t="inlineStr"/>
+      <c r="E86" s="7" t="inlineStr"/>
+      <c r="F86" s="7" t="inlineStr"/>
+      <c r="G86" s="7" t="inlineStr"/>
       <c r="H86" s="6" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="8" t="n"/>
-      <c r="B87" s="8" t="n"/>
+      <c r="A87" s="9" t="n"/>
+      <c r="B87" s="9" t="n"/>
       <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Budget control — contingency</t>
         </is>
       </c>
-      <c r="D87" s="4" t="inlineStr"/>
-      <c r="E87" s="4" t="inlineStr"/>
-      <c r="F87" s="4" t="inlineStr"/>
-      <c r="G87" s="4" t="inlineStr"/>
+      <c r="D87" s="7" t="inlineStr"/>
+      <c r="E87" s="7" t="inlineStr"/>
+      <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="7" t="inlineStr"/>
       <c r="H87" s="6" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="9" t="n">
+      <c r="A88" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B88" s="10" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>Closeout &amp; Punch List</t>
         </is>
       </c>
-      <c r="C88" s="11" t="inlineStr">
+      <c r="C88" s="10" t="inlineStr">
         <is>
           <t>Deficiency tracking</t>
         </is>
       </c>
-      <c r="D88" s="9" t="inlineStr"/>
-      <c r="E88" s="9" t="inlineStr"/>
-      <c r="F88" s="9" t="inlineStr"/>
-      <c r="G88" s="9" t="inlineStr"/>
-      <c r="H88" s="11" t="inlineStr"/>
+      <c r="D88" s="11" t="inlineStr"/>
+      <c r="E88" s="11" t="inlineStr"/>
+      <c r="F88" s="11" t="inlineStr"/>
+      <c r="G88" s="11" t="inlineStr"/>
+      <c r="H88" s="10" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="7" t="n"/>
-      <c r="B89" s="7" t="n"/>
-      <c r="C89" s="11" t="inlineStr">
+      <c r="A89" s="8" t="n"/>
+      <c r="B89" s="8" t="n"/>
+      <c r="C89" s="10" t="inlineStr">
         <is>
           <t>Warranty management</t>
         </is>
       </c>
-      <c r="D89" s="9" t="inlineStr"/>
-      <c r="E89" s="9" t="inlineStr"/>
-      <c r="F89" s="9" t="inlineStr"/>
-      <c r="G89" s="9" t="inlineStr"/>
-      <c r="H89" s="11" t="inlineStr"/>
+      <c r="D89" s="11" t="inlineStr"/>
+      <c r="E89" s="11" t="inlineStr"/>
+      <c r="F89" s="11" t="inlineStr"/>
+      <c r="G89" s="11" t="inlineStr"/>
+      <c r="H89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="8" t="n"/>
-      <c r="B90" s="8" t="n"/>
-      <c r="C90" s="11" t="inlineStr">
+      <c r="A90" s="9" t="n"/>
+      <c r="B90" s="9" t="n"/>
+      <c r="C90" s="10" t="inlineStr">
         <is>
           <t>Readiness for phased opening</t>
         </is>
       </c>
-      <c r="D90" s="9" t="inlineStr"/>
-      <c r="E90" s="9" t="inlineStr"/>
-      <c r="F90" s="9" t="inlineStr"/>
-      <c r="G90" s="9" t="inlineStr"/>
-      <c r="H90" s="11" t="inlineStr"/>
+      <c r="D90" s="11" t="inlineStr"/>
+      <c r="E90" s="11" t="inlineStr"/>
+      <c r="F90" s="11" t="inlineStr"/>
+      <c r="G90" s="11" t="inlineStr"/>
+      <c r="H90" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:H90"/>
@@ -2045,17 +2045,17 @@
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>E — Secondary Responsibility – Owner PDG</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Owner PDG</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Owner PDG supporting / backup role: reviews, contributes, or covers when the lead is unavailable.</t>
         </is>
@@ -2079,17 +2079,17 @@
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>G — Secondary Responsibility – DNC Developer</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>DNC Developer</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>DNC Developer supporting / backup role: assists or steps in behind the developer lead.</t>
         </is>
@@ -2122,17 +2122,17 @@
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Cost, Change Orders, Contracts</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>2. Budget / Cost Control
 4. Change Management
@@ -2160,17 +2160,17 @@
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Person 3</t>
         </is>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Quality, Design, Commissioning</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>5. Scope Control
 6. Design Coordination &amp; Completion
@@ -2199,17 +2199,17 @@
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Person 5</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Site Operations — MEP, FA, FP, Security</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>12. MEP &amp; Systems Integration
 14. Casino-Specific Systems / Interface

</xml_diff>